<commit_message>
Auto backup 2026-07-02 02:35:01
</commit_message>
<xml_diff>
--- a/SwissTechSaqib/Swiss Tech Files 2025/Ledgers 2025/Fedex Labels/05 FedEx Labels Report June 2026.xlsx
+++ b/SwissTechSaqib/Swiss Tech Files 2025/Ledgers 2025/Fedex Labels/05 FedEx Labels Report June 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\SwissTechSaqib\Swiss Tech Files 2025\Ledgers 2025\Fedex Labels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3157456A-0CAE-4E2C-A488-89F9CE88BF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F577DB6A-3E03-4E02-8DCC-CC171B89393D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Swiss Tech LLC Labels" sheetId="7" r:id="rId1"/>
@@ -116,7 +116,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -132,6 +132,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -181,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -220,6 +226,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="15" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,16 +554,16 @@
       <c r="D2" s="6"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
+      <c r="A3" s="14">
         <v>46184</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="15">
         <v>872959357726</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="16">
         <v>89.69</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="17" t="s">
         <v>2</v>
       </c>
     </row>
@@ -629,36 +651,36 @@
       <c r="D16" s="11"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="10">
+      <c r="A20" s="18">
         <v>46175</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="16">
         <v>1833.25</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="19" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="10">
+      <c r="A22" s="18">
         <v>46195</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22" s="16">
         <v>2472.85</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="19" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>